<commit_message>
Expand to 40 blog topics (Focus 1 + Focus 2), update field names in all scripts
</commit_message>
<xml_diff>
--- a/cavea_automation/blog_tracking.xlsx
+++ b/cavea_automation/blog_tracking.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blog Topics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blog Tracking" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,13 +26,19 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00C4A24E"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -44,20 +50,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002D2D2D"/>
-        <bgColor rgb="002D2D2D"/>
+        <fgColor rgb="001A1A2E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A3D1A"/>
-        <bgColor rgb="001A3D1A"/>
+        <fgColor rgb="00C6A969"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="003D3D1A"/>
-        <bgColor rgb="003D3D1A"/>
+        <fgColor rgb="002D2D44"/>
       </patternFill>
     </fill>
   </fills>
@@ -70,18 +73,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00555555"/>
-      </left>
-      <right style="thin">
-        <color rgb="00555555"/>
-      </right>
-      <top style="thin">
-        <color rgb="00555555"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00555555"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -92,11 +87,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -464,16 +459,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1141,6 +1136,626 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Investeren in wijn</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Investeren in Wijn: Is dit nog Winstgevend in 2025? (Marktanalyse)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>investeren-in-wijn-is-dit-nog-winstgevend-in-2025-marktanaly</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Wijnmarkt analyse</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Wijn als belegging</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Wijn als Belegging: Hoe Waardebepaling werkt en wat de Grootste Risico's zijn</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>wijn-als-belegging-hoe-waardebepaling-werkt-en-wat-de-groots</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Waardebepaling en risico's</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Exclusieve wijn kopen</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>5 Tips voor het Kopen van Exclusieve Wijn met Gegarandeerde Herkomst</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>5-tips-voor-het-kopen-van-exclusieve-wijn-met-gegarandeerde</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Herkomst en zeldzaamheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>En Primeur kopen</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>En Primeur Kopen: Welke Topregio's en Jaargangen moet je in de gaten houden?</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>en-primeur-kopen-welke-topregios-en-jaargangen-moet-je-in-de</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Topregio's en jaargangen</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Sassicaia kopen</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>De Prijsontwikkeling van Sassicaia: Waar en Hoe koop je authentieke flessen?</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>de-prijsontwikkeling-van-sassicaia-waar-en-hoe-koop-je-authe</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Prijsontwikkeling en authenticiteit</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Allocatiewijn</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Allocatiewijn en Relatiebeheer: De Sleutel tot de Meest Exclusieve Wijnen</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>allocatiewijn-en-relatiebeheer-de-sleutel-tot-de-meest-exclu</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Bouwen van relaties</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Wijnportefeuille</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Je Wijnportefeuille Beheren en Optimaliseren: Focus op Liquiditeit en Groei</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>je-wijnportefeuille-beheren-en-optimaliseren-focus-op-liquid</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Beheer en liquiditeit</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Grand Cru Classé kopen</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>De Beste Grand Cru Classé van de Linker- en Rechteroever om Vandaag te Kopen</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>de-beste-grand-cru-classe-van-de-linker-en-rechteroever-om-v</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Topchâteaux en bewaarpotentieel</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Waardevaste wijnen</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Waardevaste Wijnen Buiten Bordeaux: De Ontdekking van Rendabele Regio's</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>waardevaste-wijnen-buiten-bordeaux-de-ontdekking-van-rendabe</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Alternatieven voor Bordeaux</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Bewaarpotentieel</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Maximale Houdbaarheid: De Perfecte Omstandigheden voor Wijn met Hoog Bewaarpotentieel</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>maximale-houdbaarheid-de-perfecte-omstandigheden-voor-wijn-m</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Optimale opslag</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Beste wijn om in te investeren 2025</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>De Opkomende Wijnregio's en Nieuwe Namen met het Hoogste Investeringspotentieel in 2025</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>de-opkomende-wijnregios-en-nieuwe-namen-met-het-hoogste-inve</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Nieuwe en opkomende wijnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>BTW vrij wijn kopen en opslaan</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>BTW Vrij Wijn Kopen: Zo Kies je een Gecertificeerde en Beveiligde Opslagplaats</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>btw-vrij-wijn-kopen-zo-kies-je-een-gecertificeerde-en-beveil</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Gecertificeerde opslag</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Welke wijnen stijgen in waarde</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Een Historische Analyse van Wijn Waardestijging: De 10 Grootste Stijgers van de Afgelopen 10 Jaar</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>een-historische-analyse-van-wijn-waardestijging-de-10-groots</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Historische analyse</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Gemiddeld rendement op wijninvestering</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Het Risico-Rendement Profiel van Wijninvestering: Wat je Realistisch kunt Verwachten</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>het-risico-rendement-profiel-van-wijninvestering-wat-je-real</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Risico-rendement profiel</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Toegang tot exclusieve wijn allocaties</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Exclusieve Wijn Allocaties: De Top Internationale Programma's waar je Lid van moet Worden</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>exclusieve-wijn-allocaties-de-top-internationale-programmas</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Internationale allocatieprogramma's</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Investeren in Grand Cru Classé Bordeaux</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Grand Cru Classé Bordeaux: De Beste Châteaux Selecteren voor je Investeringsportefeuille</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>grand-cru-classe-bordeaux-de-beste-chateaux-selecteren-voor</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Kwaliteitsselectie</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Sassicaia Tenuta San Guido kopen</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Sassicaia Kopen: Direct bij de Wijnboer of Via een Veilingshuis? Alle Opties</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>sassicaia-kopen-direct-bij-de-wijnboer-of-via-een-veilingshu</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Directe aankoop en veiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Hulp bij wijnportefeuille samenstellen</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Je Wijnportefeuille Professioneel Laten Samenstellen: Wanneer en Hoe Expertise Inschakelen</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>je-wijnportefeuille-professioneel-laten-samenstellen-wanneer</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Expertise inschakelen</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Wijn kopen in de voorverkoop (En Primeur)</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>En Primeur Wijn Kopen: Hoe Groot is het Potentiële Prijsverschil en Wat is de Gemiddelde ROI?</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>en-primeur-wijn-kopen-hoe-groot-is-het-potentiele-prijsversc</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Prijsverschil en ROI</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Rode bewaarwijn met potentieel</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Top Rode Bewaarwijn met Gegarandeerd Potentieel: Een Gedetailleerd Rijpingsschema</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>top-rode-bewaarwijn-met-gegarandeerd-potentieel-een-gedetail</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Opslag en rijpingsschema</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Update blog topics status
</commit_message>
<xml_diff>
--- a/cavea_automation/blog_tracking.xlsx
+++ b/cavea_automation/blog_tracking.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blog Tracking" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Blog Topics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,19 +26,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
-      <sz val="10"/>
+      <color rgb="00C4A24E"/>
     </font>
   </fonts>
   <fills count="5">
@@ -50,17 +44,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A1A2E"/>
+        <fgColor rgb="002D2D2D"/>
+        <bgColor rgb="002D2D2D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6A969"/>
+        <fgColor rgb="001A3D1A"/>
+        <bgColor rgb="001A3D1A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002D2D44"/>
+        <fgColor rgb="003D3D1A"/>
+        <bgColor rgb="003D3D1A"/>
       </patternFill>
     </fill>
   </fills>
@@ -73,10 +70,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00555555"/>
+      </left>
+      <right style="thin">
+        <color rgb="00555555"/>
+      </right>
+      <top style="thin">
+        <color rgb="00555555"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00555555"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -87,11 +92,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -464,11 +469,11 @@
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -597,12 +602,16 @@
           <t>exclusieve-wijn-kopen-beste-adressen</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>USED</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Via welke kanalen</t>

</xml_diff>